<commit_message>
add salary matrix db table design
</commit_message>
<xml_diff>
--- a/Documents/Online Job Offer System - User Stories V2.xlsx
+++ b/Documents/Online Job Offer System - User Stories V2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unitedlaboratoriesinc-my.sharepoint.com/personal/rmlee_unilab_com_ph/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="8_{ACE7F87D-810E-41ED-BE92-06FDE3D8E5EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F121A1E6-D985-480B-9DAF-F675C7BADCE3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC247D6-13A3-482C-A8C9-2AE6A7C33379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Epic_Overview" sheetId="1" r:id="rId1"/>
@@ -3590,7 +3590,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3610,6 +3610,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -3643,7 +3655,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3738,6 +3750,15 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4214,7 +4235,7 @@
       <c r="B2" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="34" t="s">
         <v>35</v>
       </c>
       <c r="D2" s="16" t="s">
@@ -4261,7 +4282,7 @@
       <c r="B3" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="34" t="s">
         <v>35</v>
       </c>
       <c r="D3" s="18" t="s">
@@ -4308,7 +4329,7 @@
       <c r="B4" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="34" t="s">
         <v>35</v>
       </c>
       <c r="D4" s="16" t="s">
@@ -4355,7 +4376,7 @@
       <c r="B5" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="35" t="s">
         <v>67</v>
       </c>
       <c r="D5" s="22" t="s">
@@ -4402,7 +4423,7 @@
       <c r="B6" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="35" t="s">
         <v>79</v>
       </c>
       <c r="D6" s="25" t="s">
@@ -4449,7 +4470,7 @@
       <c r="B7" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="35" t="s">
         <v>91</v>
       </c>
       <c r="D7" s="22" t="s">
@@ -4496,7 +4517,7 @@
       <c r="B8" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="35" t="s">
         <v>104</v>
       </c>
       <c r="D8" s="25" t="s">
@@ -4543,7 +4564,7 @@
       <c r="B9" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="34" t="s">
         <v>104</v>
       </c>
       <c r="D9" s="18" t="s">
@@ -4590,7 +4611,7 @@
       <c r="B10" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="34" t="s">
         <v>104</v>
       </c>
       <c r="D10" s="16" t="s">
@@ -4637,7 +4658,7 @@
       <c r="B11" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="34" t="s">
         <v>140</v>
       </c>
       <c r="D11" s="18" t="s">
@@ -4684,7 +4705,7 @@
       <c r="B12" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="35" t="s">
         <v>140</v>
       </c>
       <c r="D12" s="25" t="s">
@@ -4731,7 +4752,7 @@
       <c r="B13" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="34" t="s">
         <v>164</v>
       </c>
       <c r="D13" s="18" t="s">
@@ -4772,13 +4793,13 @@
       </c>
     </row>
     <row r="14" spans="1:15" s="23" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="35" t="s">
         <v>175</v>
       </c>
       <c r="B14" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="35" t="s">
         <v>176</v>
       </c>
       <c r="D14" s="25" t="s">
@@ -4819,13 +4840,13 @@
       </c>
     </row>
     <row r="15" spans="1:15" s="23" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="36" t="s">
         <v>187</v>
       </c>
       <c r="B15" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="35" t="s">
         <v>188</v>
       </c>
       <c r="D15" s="22" t="s">
@@ -4872,7 +4893,7 @@
       <c r="B16" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="34" t="s">
         <v>201</v>
       </c>
       <c r="D16" s="16" t="s">
@@ -4919,7 +4940,7 @@
       <c r="B17" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="34" t="s">
         <v>213</v>
       </c>
       <c r="D17" s="18" t="s">
@@ -4966,7 +4987,7 @@
       <c r="B18" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="34" t="s">
         <v>225</v>
       </c>
       <c r="D18" s="16" t="s">
@@ -5013,7 +5034,7 @@
       <c r="B19" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="34" t="s">
         <v>238</v>
       </c>
       <c r="D19" s="18" t="s">
@@ -5060,7 +5081,7 @@
       <c r="B20" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="34" t="s">
         <v>251</v>
       </c>
       <c r="D20" s="16" t="s">
@@ -5107,7 +5128,7 @@
       <c r="B21" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="35" t="s">
         <v>263</v>
       </c>
       <c r="D21" s="25" t="s">
@@ -5154,7 +5175,7 @@
       <c r="B22" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="35" t="s">
         <v>263</v>
       </c>
       <c r="D22" s="25" t="s">

</xml_diff>

<commit_message>
end of shift commit
</commit_message>
<xml_diff>
--- a/Documents/Online Job Offer System - User Stories V2.xlsx
+++ b/Documents/Online Job Offer System - User Stories V2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC247D6-13A3-482C-A8C9-2AE6A7C33379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC4BE9B3-E915-464F-8BF9-7F62BEB37968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3590,7 +3590,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3615,12 +3615,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3758,7 +3752,7 @@
     <xf numFmtId="0" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>